<commit_message>
Complete Sprint 4 Streamlit Dashboard
</commit_message>
<xml_diff>
--- a/data/raw/analysis.xlsx
+++ b/data/raw/analysis.xlsx
@@ -1,15 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analysis'!$A$2:$F$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +27,47 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +75,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,52 +472,701 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bluestock Fintech — Nifty 100  |  Analysis  |  20 records</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>remarks</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Good</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>compounded_sales_growth</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>compounded_profit_growth</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>stock_price_cagr</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>roe</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Average</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>10 Years: 21%</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>10 Years: 22%</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>10 Years:     15%</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>10 Years:     17%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Excellent</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:       24%</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:            6%</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     5 Years:       8%</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>5 Years          14%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>3 Years:       17%</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>3 Years:            9%</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     3 Years:       7%</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>3 Years:         13%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>TTM:            43%</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>TTM:                 18%</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     1 Year:         -2%</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Last Year:      12%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10 Years:     11%             </t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>10 Years:          9%</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    10 Years:      14%</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>10 Years:       40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Years:       10%             </t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:            8%</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      5 Years:      16%</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:          44%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Years:       14%             </t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>3 Years:            12%</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      3 Years:      8%</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>3 Years:          47%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TTM:            5%             </t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>TTM:                 8%</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      1 Year:       16%</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Last Year:       52%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>10 Years:     8%</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>10 Years:          3%</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    10 Years:     12%</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>10 Years:        18%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:       9%</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:            4%</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      5 Years:     20%</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:          17%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>3 Years:      13%</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>3 Years:            0%</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      3 Years:      -1%</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>3 Years:          17%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:       22%</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:           23%</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      5 Years:       8%</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>5 Years:       17%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>TTM:           -3%</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>TTM:                 1%</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      1 Year:       39%</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Last Year:       14%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>3 Years:       30%</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>3 Years:           26%</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      3 Years:       8%</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>3 Years:       17%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>TTM:            47%</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>TTM:                27%</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      1 Year:        13%</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Last Year:    17%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>10 Years:     12%</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>10 Years:         9%</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     10 Years:     15%</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>10 Years:      27%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>5 Years:       13%</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>5 Years:           11%</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       5 Years:     22%</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>5 Years:        29%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>3 Years:       5%</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>3 Years:           10%</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       3 Years:     4%</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>3 Years:        31%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>TTM:            3%</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>TTM:                 8%</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       1 Year:       27%</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Last Year:     32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>10 Years:     23%</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>10 Years:          9%</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    10 Years:      9%</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>10 Years:      16%</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:F2"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>